<commit_message>
Update atlas coordinates from user-reviewed project list (56 locations; flag CSP mismatch)
</commit_message>
<xml_diff>
--- a/data/proyectos.xlsx
+++ b/data/proyectos.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="1" r:id="Rc414f05b57af447c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen_42" sheetId="2" r:id="R81f30fbb061247ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="3" r:id="R609b3072b2f44126"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="1" r:id="Rf99a7e57f13249d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen_42" sheetId="2" r:id="R57eb53133f3d4543"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="3" r:id="Rf3b3ab56fa7b453e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -87,14 +87,14 @@
   <x:dxfs count="2">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF5EA"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D9"/>
         </x:patternFill>
       </x:fill>
@@ -440,11 +440,11 @@
       <x:c r="G2" t="str">
         <x:v>San José</x:v>
       </x:c>
-      <x:c r="H2" s="10" t="str">
-        <x:v>9.9281</x:v>
-      </x:c>
-      <x:c r="I2" s="10" t="str">
-        <x:v>-84.0907</x:v>
+      <x:c r="H2" s="10" t="n">
+        <x:v>9.952180991628238</x:v>
+      </x:c>
+      <x:c r="I2" s="10" t="n">
+        <x:v>-84.09912805674576</x:v>
       </x:c>
       <x:c r="J2" t="str">
         <x:v>2016</x:v>
@@ -479,7 +479,7 @@
       </x:c>
       <x:c r="U2" s="8" t="str"/>
       <x:c r="V2" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=AyA%20%E2%80%93%20Direcci%C3%B3n%20de%20Mejoramiento%20de%20Sistemas%2C%20San%20Jos%C3%A9%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.95218099162824%2C-84.09912805674576</x:v>
       </x:c>
       <x:c r="W2" t="str"/>
       <x:c r="X2" s="8" t="str">
@@ -492,13 +492,13 @@
         <x:v>Optimización metropolitana y dirección de equipos técnicos</x:v>
       </x:c>
       <x:c r="AA2" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB2" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC2" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -523,11 +523,11 @@
       <x:c r="G3" t="str">
         <x:v>San José</x:v>
       </x:c>
-      <x:c r="H3" s="10" t="str">
-        <x:v>9.934</x:v>
-      </x:c>
-      <x:c r="I3" s="10" t="str">
-        <x:v>-84.076</x:v>
+      <x:c r="H3" s="10" t="n">
+        <x:v>9.933137472963232</x:v>
+      </x:c>
+      <x:c r="I3" s="10" t="n">
+        <x:v>-84.0435391275236</x:v>
       </x:c>
       <x:c r="J3" t="str">
         <x:v>2018</x:v>
@@ -560,7 +560,7 @@
       </x:c>
       <x:c r="U3" s="8" t="str"/>
       <x:c r="V3" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Universidad%20Latina%2C%20San%20Jos%C3%A9%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93313747296323%2C-84.04353912752360</x:v>
       </x:c>
       <x:c r="W3" t="str"/>
       <x:c r="X3" s="8" t="str">
@@ -573,13 +573,13 @@
         <x:v>Mecánica de fluidos e ingeniería sanitaria</x:v>
       </x:c>
       <x:c r="AA3" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB3" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -604,11 +604,11 @@
       <x:c r="G4" t="str">
         <x:v>San José</x:v>
       </x:c>
-      <x:c r="H4" s="10" t="str">
-        <x:v>9.9281</x:v>
-      </x:c>
-      <x:c r="I4" s="10" t="str">
-        <x:v>-84.0907</x:v>
+      <x:c r="H4" s="10" t="n">
+        <x:v>9.946063562539855</x:v>
+      </x:c>
+      <x:c r="I4" s="10" t="n">
+        <x:v>-84.19570527219565</x:v>
       </x:c>
       <x:c r="J4" t="str">
         <x:v>2013</x:v>
@@ -643,7 +643,7 @@
       </x:c>
       <x:c r="U4" s="8" t="str"/>
       <x:c r="V4" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Santos%20CMI%2C%20San%20Jos%C3%A9%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.94606356253986%2C-84.19570527219565</x:v>
       </x:c>
       <x:c r="W4" t="str"/>
       <x:c r="X4" s="8" t="str">
@@ -656,13 +656,13 @@
         <x:v>Diseño de infraestructura para proyectos energéticos</x:v>
       </x:c>
       <x:c r="AA4" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB4" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC4" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -687,11 +687,11 @@
       <x:c r="G5" t="str">
         <x:v>San Rafael de Oreamuno</x:v>
       </x:c>
-      <x:c r="H5" s="10" t="str">
-        <x:v>9.868</x:v>
-      </x:c>
-      <x:c r="I5" s="10" t="str">
-        <x:v>-83.905</x:v>
+      <x:c r="H5" s="10" t="n">
+        <x:v>9.868918971436047</x:v>
+      </x:c>
+      <x:c r="I5" s="10" t="n">
+        <x:v>-83.9042102677281</x:v>
       </x:c>
       <x:c r="J5" t="str">
         <x:v>2015</x:v>
@@ -728,7 +728,7 @@
       </x:c>
       <x:c r="U5" s="8" t="str"/>
       <x:c r="V5" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Municipalidad%20de%20Oreamuno%2C%20San%20Rafael%20de%20Oreamuno%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.86891897143605%2C-83.90421026772810</x:v>
       </x:c>
       <x:c r="W5" t="str"/>
       <x:c r="X5" s="8" t="str">
@@ -741,13 +741,13 @@
         <x:v>Administración vial y proyectos cantonales</x:v>
       </x:c>
       <x:c r="AA5" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB5" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC5" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -772,11 +772,11 @@
       <x:c r="G6" t="str">
         <x:v>San José</x:v>
       </x:c>
-      <x:c r="H6" s="10" t="str">
-        <x:v>9.9281</x:v>
-      </x:c>
-      <x:c r="I6" s="10" t="str">
-        <x:v>-84.0907</x:v>
+      <x:c r="H6" s="10" t="n">
+        <x:v>9.96645430288732</x:v>
+      </x:c>
+      <x:c r="I6" s="10" t="n">
+        <x:v>-84.36234267645101</x:v>
       </x:c>
       <x:c r="J6" t="str">
         <x:v>2015</x:v>
@@ -811,7 +811,7 @@
       </x:c>
       <x:c r="U6" s="8" t="str"/>
       <x:c r="V6" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=SCH%20Consultor%C3%ADa%20y%20Construcci%C3%B3n%2C%20San%20Jos%C3%A9%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.96645430288732%2C-84.36234267645101</x:v>
       </x:c>
       <x:c r="W6" t="str"/>
       <x:c r="X6" s="8" t="str">
@@ -824,13 +824,13 @@
         <x:v>Gestión de remodelaciones industriales</x:v>
       </x:c>
       <x:c r="AA6" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB6" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC6" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -855,11 +855,11 @@
       <x:c r="G7" t="str">
         <x:v>San José</x:v>
       </x:c>
-      <x:c r="H7" s="10" t="str">
-        <x:v>9.9281</x:v>
-      </x:c>
-      <x:c r="I7" s="10" t="str">
-        <x:v>-84.0907</x:v>
+      <x:c r="H7" s="10" t="n">
+        <x:v>9.939017744116914</x:v>
+      </x:c>
+      <x:c r="I7" s="10" t="n">
+        <x:v>-84.05919790858356</x:v>
       </x:c>
       <x:c r="J7" t="str">
         <x:v>2012</x:v>
@@ -894,7 +894,7 @@
       </x:c>
       <x:c r="U7" s="8" t="str"/>
       <x:c r="V7" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=FUPROVI%2C%20San%20Jos%C3%A9%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93901774411691%2C-84.05919790858356</x:v>
       </x:c>
       <x:c r="W7" t="str"/>
       <x:c r="X7" s="8" t="str">
@@ -907,13 +907,13 @@
         <x:v>Supervisión de infraestructura residencial</x:v>
       </x:c>
       <x:c r="AA7" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB7" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -938,11 +938,11 @@
       <x:c r="G8" t="str">
         <x:v>Belén / Puente Mulas</x:v>
       </x:c>
-      <x:c r="H8" s="10" t="str">
-        <x:v>9.979</x:v>
-      </x:c>
-      <x:c r="I8" s="10" t="str">
-        <x:v>-84.177</x:v>
+      <x:c r="H8" s="10" t="n">
+        <x:v>9.972706975052512</x:v>
+      </x:c>
+      <x:c r="I8" s="10" t="n">
+        <x:v>-84.18383232588455</x:v>
       </x:c>
       <x:c r="J8" t="str">
         <x:v>2025</x:v>
@@ -979,7 +979,7 @@
         <x:v>https://www.santaanahoy.com/m%C3%A1s-agua-para-m%C3%A1s-personas-de-la-gam</x:v>
       </x:c>
       <x:c r="V8" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Fuente%20Zamora%20Grupo%20Pedregal%20Puente%20Mulas%20Bel%C3%A9n%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.97270697505251%2C-84.18383232588455</x:v>
       </x:c>
       <x:c r="W8" t="str"/>
       <x:c r="X8" s="8" t="str">
@@ -992,13 +992,13 @@
         <x:v>Apoyo a puesta en marcha, medición y análisis de caudal; evaluación del aporte de la fuente y su efecto sobre disponibilidad y estabilidad del sistema.</x:v>
       </x:c>
       <x:c r="AA8" s="8" t="str">
-        <x:v>Referencia Belén-Puente Mulas; sitio físico por confirmar</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB8" s="8" t="str">
         <x:v>turn6search563; turn6search455</x:v>
       </x:c>
       <x:c r="AC8" t="str">
-        <x:v>Por verificar</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1023,11 +1023,11 @@
       <x:c r="G9" t="str">
         <x:v>Bebedero</x:v>
       </x:c>
-      <x:c r="H9" s="10" t="str">
-        <x:v>10.378</x:v>
-      </x:c>
-      <x:c r="I9" s="10" t="str">
-        <x:v>-85.196</x:v>
+      <x:c r="H9" s="10" t="n">
+        <x:v>10.459032589649608</x:v>
+      </x:c>
+      <x:c r="I9" s="10" t="n">
+        <x:v>-85.0930094542223</x:v>
       </x:c>
       <x:c r="J9" t="str">
         <x:v>2016</x:v>
@@ -1064,7 +1064,7 @@
       </x:c>
       <x:c r="U9" s="8" t="str"/>
       <x:c r="V9" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Planta%20potabilizadora%20Ca%C3%B1as-Bebedero%2C%20Bebedero%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=10.45903258964961%2C-85.09300945422230</x:v>
       </x:c>
       <x:c r="W9" t="str"/>
       <x:c r="X9" s="8" t="str">
@@ -1077,13 +1077,13 @@
         <x:v>Actualización de matriz del proyecto, seguimiento de información para Mesa Chorotega, coordinación con PMO e incorporación de estado y programación del proyecto.</x:v>
       </x:c>
       <x:c r="AA9" s="8" t="str">
-        <x:v>Referente poblacional de Cañas-Bebedero; no indica la planta</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB9" s="8" t="str">
         <x:v>turn6search493</x:v>
       </x:c>
       <x:c r="AC9" t="str">
-        <x:v>Por verificar</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1108,11 +1108,11 @@
       <x:c r="G10" t="str">
         <x:v>Sardinal</x:v>
       </x:c>
-      <x:c r="H10" s="10" t="str">
-        <x:v>10.527</x:v>
-      </x:c>
-      <x:c r="I10" s="10" t="str">
-        <x:v>-85.673</x:v>
+      <x:c r="H10" s="10" t="n">
+        <x:v>10.519669341620059</x:v>
+      </x:c>
+      <x:c r="I10" s="10" t="n">
+        <x:v>-85.6533411785515</x:v>
       </x:c>
       <x:c r="J10" t="str">
         <x:v>2016</x:v>
@@ -1149,7 +1149,7 @@
       </x:c>
       <x:c r="U10" s="8" t="str"/>
       <x:c r="V10" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Acueducto%20Sardinal%E2%80%93El%20Coco%E2%80%93Ocotal%2C%20Sardinal%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=10.51966934162006%2C-85.65334117855150</x:v>
       </x:c>
       <x:c r="W10" t="str"/>
       <x:c r="X10" s="8" t="str">
@@ -1162,13 +1162,13 @@
         <x:v>Sistema de pozos y almacenamiento</x:v>
       </x:c>
       <x:c r="AA10" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB10" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC10" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1193,11 +1193,11 @@
       <x:c r="G11" t="str">
         <x:v>Tamarindo</x:v>
       </x:c>
-      <x:c r="H11" s="10" t="str">
-        <x:v>10.299</x:v>
-      </x:c>
-      <x:c r="I11" s="10" t="str">
-        <x:v>-85.84</x:v>
+      <x:c r="H11" s="10" t="n">
+        <x:v>10.365783983782595</x:v>
+      </x:c>
+      <x:c r="I11" s="10" t="n">
+        <x:v>-85.69756378618713</x:v>
       </x:c>
       <x:c r="J11" t="str">
         <x:v>2016</x:v>
@@ -1234,7 +1234,7 @@
       </x:c>
       <x:c r="U11" s="8" t="str"/>
       <x:c r="V11" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Acueducto%20regional%20Nimboyores%2C%20Tamarindo%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=10.36578398378260%2C-85.69756378618713</x:v>
       </x:c>
       <x:c r="W11" t="str"/>
       <x:c r="X11" s="8" t="str">
@@ -1247,13 +1247,13 @@
         <x:v>Conducción regional y etapas de infraestructura</x:v>
       </x:c>
       <x:c r="AA11" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB11" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC11" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1278,11 +1278,11 @@
       <x:c r="G12" t="str">
         <x:v>Alajuelita</x:v>
       </x:c>
-      <x:c r="H12" s="10" t="str">
-        <x:v>9.899</x:v>
-      </x:c>
-      <x:c r="I12" s="10" t="str">
-        <x:v>-84.101</x:v>
+      <x:c r="H12" s="10" t="n">
+        <x:v>9.928226400465373</x:v>
+      </x:c>
+      <x:c r="I12" s="10" t="n">
+        <x:v>-84.08909995879816</x:v>
       </x:c>
       <x:c r="J12" t="str">
         <x:v>2024</x:v>
@@ -1319,7 +1319,7 @@
       </x:c>
       <x:c r="U12" s="8" t="str"/>
       <x:c r="V12" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Campa%C3%B1as%20de%20sectorizaci%C3%B3n%20GAM%2C%20Alajuelita%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.92822640046537%2C-84.08909995879816</x:v>
       </x:c>
       <x:c r="W12" t="str"/>
       <x:c r="X12" s="8" t="str">
@@ -1332,13 +1332,13 @@
         <x:v>Elaboración y seguimiento de planes e informes técnicos sobre sectorización, presiones, fugas, continuidad, cronogramas y acciones de corto, mediano y largo plazo.</x:v>
       </x:c>
       <x:c r="AA12" s="8" t="str">
-        <x:v>Campañas en varios distritos; punto de referencia representativo</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB12" s="8" t="str">
         <x:v>turn6search447; turn6search497; turn2search369</x:v>
       </x:c>
       <x:c r="AC12" t="str">
-        <x:v>Por verificar</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1363,11 +1363,11 @@
       <x:c r="G13" t="str">
         <x:v>San José</x:v>
       </x:c>
-      <x:c r="H13" s="10" t="str">
-        <x:v>9.9281</x:v>
-      </x:c>
-      <x:c r="I13" s="10" t="str">
-        <x:v>-84.0907</x:v>
+      <x:c r="H13" s="10" t="n">
+        <x:v>9.939163048006971</x:v>
+      </x:c>
+      <x:c r="I13" s="10" t="n">
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J13" t="str">
         <x:v>2025</x:v>
@@ -1404,7 +1404,7 @@
       </x:c>
       <x:c r="U13" s="8" t="str"/>
       <x:c r="V13" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=PRAGAM%20%E2%80%93%20planificaci%C3%B3n%20metropolitana%2C%20San%20Jos%C3%A9%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W13" t="str"/>
       <x:c r="X13" s="8" t="str">
@@ -1417,13 +1417,13 @@
         <x:v>Apoyo en mapa/visor de proyectos, etapas del ciclo de inversión, cronogramas, evaluación de alternativas y articulación de iniciativas de acción inmediata, corto, mediano y largo plazo.</x:v>
       </x:c>
       <x:c r="AA13" s="8" t="str">
-        <x:v>Programa multiproyecto; referencia San José sin ubicación única</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB13" s="8" t="str">
         <x:v>turn6search443; turn6search446; turn6search433</x:v>
       </x:c>
       <x:c r="AC13" t="str">
-        <x:v>Por verificar</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1448,11 +1448,11 @@
       <x:c r="G14" t="str">
         <x:v>San José</x:v>
       </x:c>
-      <x:c r="H14" s="10" t="str">
-        <x:v>9.9281</x:v>
-      </x:c>
-      <x:c r="I14" s="10" t="str">
-        <x:v>-84.0907</x:v>
+      <x:c r="H14" s="10" t="n">
+        <x:v>9.939163048006971</x:v>
+      </x:c>
+      <x:c r="I14" s="10" t="n">
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J14" t="str">
         <x:v>2026</x:v>
@@ -1485,7 +1485,7 @@
       </x:c>
       <x:c r="U14" s="8" t="str"/>
       <x:c r="V14" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Visor%20de%20capacidad%20h%C3%ADdrica%20GAM%2C%20San%20Jos%C3%A9%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W14" t="str"/>
       <x:c r="X14" s="8" t="str">
@@ -1498,13 +1498,13 @@
         <x:v>Visor de capacidad hídrica y datos geoespaciales</x:v>
       </x:c>
       <x:c r="AA14" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB14" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC14" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1529,11 +1529,11 @@
       <x:c r="G15" t="str">
         <x:v>San José</x:v>
       </x:c>
-      <x:c r="H15" s="10" t="str">
-        <x:v>9.9281</x:v>
-      </x:c>
-      <x:c r="I15" s="10" t="str">
-        <x:v>-84.0907</x:v>
+      <x:c r="H15" s="10" t="n">
+        <x:v>9.952180991628238</x:v>
+      </x:c>
+      <x:c r="I15" s="10" t="n">
+        <x:v>-84.09912805674576</x:v>
       </x:c>
       <x:c r="J15" t="str">
         <x:v>2026</x:v>
@@ -1566,7 +1566,7 @@
       </x:c>
       <x:c r="U15" s="8" t="str"/>
       <x:c r="V15" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Aplicativo%20de%20revisi%C3%B3n%20de%20caudal%C3%ADmetros%2C%20San%20Jos%C3%A9%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.95218099162824%2C-84.09912805674576</x:v>
       </x:c>
       <x:c r="W15" t="str"/>
       <x:c r="X15" s="8" t="str">
@@ -1579,13 +1579,13 @@
         <x:v>Aplicación de seguimiento integrando GIS y revisión de equipos</x:v>
       </x:c>
       <x:c r="AA15" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB15" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC15" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1610,11 +1610,11 @@
       <x:c r="G16" t="str">
         <x:v>Talagante (CMPC Tissue)</x:v>
       </x:c>
-      <x:c r="H16" s="10" t="str">
-        <x:v>-33.7055</x:v>
-      </x:c>
-      <x:c r="I16" s="10" t="str">
-        <x:v>-70.93637</x:v>
+      <x:c r="H16" s="10" t="n">
+        <x:v>-33.704037227913844</x:v>
+      </x:c>
+      <x:c r="I16" s="10" t="n">
+        <x:v>-70.93548034522583</x:v>
       </x:c>
       <x:c r="J16" t="str">
         <x:v>2013</x:v>
@@ -1653,7 +1653,7 @@
         <x:v>https://infofirma.sea.gob.cl/DocumentosSEA/MostrarDocumento?docId=f9%2F1e%2Ffce7ed7b924b34bc71ad37f6fd352bac898d</x:v>
       </x:c>
       <x:c r="V16" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Planta%20Talagante%20%E2%80%93%20Chile%2C%20Talagante%2C%20Chile</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=-33.70403722791384%2C-70.93548034522583</x:v>
       </x:c>
       <x:c r="W16" t="str"/>
       <x:c r="X16" s="8" t="str">
@@ -1666,13 +1666,13 @@
         <x:v>Aportes de diseño hidrológico y drenaje</x:v>
       </x:c>
       <x:c r="AA16" s="8" t="str">
-        <x:v>Instalación identificada mediante referencia pública; posición aproximada, sin validar predio</x:v>
+        <x:v>Coordenada suministrada y revisada por el titular; verificar correspondencia con la obra antes de atribuir una instalación física.</x:v>
       </x:c>
       <x:c r="AB16" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC16" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1697,10 +1697,10 @@
       <x:c r="G17" t="str">
         <x:v>Pecém, São Gonçalo do Amarante</x:v>
       </x:c>
-      <x:c r="H17" s="10" t="str">
+      <x:c r="H17" s="10" t="n">
         <x:v>-3.58535</x:v>
       </x:c>
-      <x:c r="I17" s="10" t="str">
+      <x:c r="I17" s="10" t="n">
         <x:v>-38.85508</x:v>
       </x:c>
       <x:c r="J17" t="str">
@@ -1753,13 +1753,13 @@
         <x:v>Participación en diseño de obras civiles y drenaje</x:v>
       </x:c>
       <x:c r="AA17" s="8" t="str">
-        <x:v>Instalación identificada mediante referencia pública; posición aproximada, sin validar predio</x:v>
+        <x:v>Revisar: la coordenada suministrada (-22.51394179581262, -44.11538570542573) no corresponde a Pecém/Ceará. Se conserva la ubicación anterior de referencia.</x:v>
       </x:c>
       <x:c r="AB17" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC17" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>PENDIENTE: coordenada suministrada incompatible con Pecém (Ceará). Mantener punto anterior hasta confirmar.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1784,11 +1784,11 @@
       <x:c r="G18" t="str">
         <x:v>Machala / Bajo Alto (por verificar)</x:v>
       </x:c>
-      <x:c r="H18" s="10" t="str">
-        <x:v>-3.258</x:v>
-      </x:c>
-      <x:c r="I18" s="10" t="str">
-        <x:v>-79.96</x:v>
+      <x:c r="H18" s="10" t="n">
+        <x:v>-3.1155096395963153</x:v>
+      </x:c>
+      <x:c r="I18" s="10" t="n">
+        <x:v>-79.8780220209804</x:v>
       </x:c>
       <x:c r="J18" t="str">
         <x:v>2013</x:v>
@@ -1827,7 +1827,7 @@
         <x:v>https://www.celec.gob.ec/electroguayas/proyectos/</x:v>
       </x:c>
       <x:c r="V18" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Central%20Machala%20Power%20%E2%80%93%20Ecuador%2C%20Machala%2C%20Ecuador</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=-3.11550963959632%2C-79.87802202098040</x:v>
       </x:c>
       <x:c r="W18" t="str"/>
       <x:c r="X18" s="8" t="str">
@@ -1840,13 +1840,13 @@
         <x:v>Participación en diseño vial e hidráulico</x:v>
       </x:c>
       <x:c r="AA18" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB18" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC18" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1871,11 +1871,11 @@
       <x:c r="G19" t="str">
         <x:v>Alajuela</x:v>
       </x:c>
-      <x:c r="H19" s="10" t="str">
-        <x:v>10.016</x:v>
-      </x:c>
-      <x:c r="I19" s="10" t="str">
-        <x:v>-84.215</x:v>
+      <x:c r="H19" s="10" t="n">
+        <x:v>9.856109080000609</x:v>
+      </x:c>
+      <x:c r="I19" s="10" t="n">
+        <x:v>-83.95586068849708</x:v>
       </x:c>
       <x:c r="J19" t="str">
         <x:v>2015</x:v>
@@ -1910,7 +1910,7 @@
       </x:c>
       <x:c r="U19" s="8" t="str"/>
       <x:c r="V19" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Gerber%E2%80%93Nestl%C3%A9%20PREVASSA%2C%20Alajuela%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.85610908000061%2C-83.95586068849708</x:v>
       </x:c>
       <x:c r="W19" t="str"/>
       <x:c r="X19" s="8" t="str">
@@ -1923,13 +1923,13 @@
         <x:v>Tratamiento de aguas y recuperación de recursos</x:v>
       </x:c>
       <x:c r="AA19" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB19" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC19" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1954,11 +1954,11 @@
       <x:c r="G20" t="str">
         <x:v>San José</x:v>
       </x:c>
-      <x:c r="H20" s="10" t="str">
-        <x:v>9.9281</x:v>
-      </x:c>
-      <x:c r="I20" s="10" t="str">
-        <x:v>-84.0907</x:v>
+      <x:c r="H20" s="10" t="n">
+        <x:v>9.920903888364052</x:v>
+      </x:c>
+      <x:c r="I20" s="10" t="n">
+        <x:v>-84.04798640395877</x:v>
       </x:c>
       <x:c r="J20" t="str">
         <x:v>2015</x:v>
@@ -1993,7 +1993,7 @@
       </x:c>
       <x:c r="U20" s="8" t="str"/>
       <x:c r="V20" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Infraestructura%20PriceSmart%2C%20San%20Jos%C3%A9%2C%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.92090388836405%2C-84.04798640395877</x:v>
       </x:c>
       <x:c r="W20" t="str"/>
       <x:c r="X20" s="8" t="str">
@@ -2006,13 +2006,13 @@
         <x:v>Soluciones de tratamiento y manejo de aguas</x:v>
       </x:c>
       <x:c r="AA20" s="8" t="str">
-        <x:v>Posición inicial de referencia; no georreferenciación de infraestructura</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB20" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC20" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2038,10 +2038,10 @@
         <x:v>San José / referencia nacional</x:v>
       </x:c>
       <x:c r="H21" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I21" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J21" t="str">
         <x:v>2017</x:v>
@@ -2076,7 +2076,7 @@
       </x:c>
       <x:c r="U21" s="8" t="str"/>
       <x:c r="V21" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Jos%C3%A9%20/%20referencia%20nacional%20Varias%20provincias%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W21" t="str"/>
       <x:c r="X21" s="8" t="str">
@@ -2089,13 +2089,13 @@
         <x:v>Revisión, recopilación, control y capitalización de inversiones; reconstrucción de antecedentes, costos, etapas, expedientes y datos de proyectos ejecutados entre 2018 y 2021.</x:v>
       </x:c>
       <x:c r="AA21" s="8" t="str">
-        <x:v>Cartera de todo el país, no existe punto único</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB21" s="8" t="str">
         <x:v>turn6search438; turn6search441; turn6search449</x:v>
       </x:c>
       <x:c r="AC21" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -2121,10 +2121,10 @@
         <x:v>Coto Brus</x:v>
       </x:c>
       <x:c r="H22" s="10" t="n">
-        <x:v>8.8855</x:v>
+        <x:v>8.821146234860828</x:v>
       </x:c>
       <x:c r="I22" s="10" t="n">
-        <x:v>-82.9412</x:v>
+        <x:v>-82.96834835171164</x:v>
       </x:c>
       <x:c r="J22" t="str">
         <x:v>2022</x:v>
@@ -2159,7 +2159,7 @@
         <x:v>https://mapcarta.com/19593780</x:v>
       </x:c>
       <x:c r="V22" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Coto%20Brus%20Coto%20Brus%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=8.82114623486083%2C-82.96834835171164</x:v>
       </x:c>
       <x:c r="W22" t="str"/>
       <x:c r="X22" s="8" t="str">
@@ -2172,13 +2172,13 @@
         <x:v>Revisión de información técnica, programación, etapa, costos estimados y financiamiento dentro del Plan de Inversiones 2022-2026 y programa BCIE 1725.</x:v>
       </x:c>
       <x:c r="AA22" s="8" t="str">
-        <x:v>Centro cantonal; Las Tablas es una referencia extensa por confirmar</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB22" s="8" t="str">
         <x:v>turn6search524</x:v>
       </x:c>
       <x:c r="AC22" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -2204,10 +2204,10 @@
         <x:v>Golfito</x:v>
       </x:c>
       <x:c r="H23" s="10" t="n">
-        <x:v>8.643</x:v>
+        <x:v>8.546361642257347</x:v>
       </x:c>
       <x:c r="I23" s="10" t="n">
-        <x:v>-83.166</x:v>
+        <x:v>-83.30926901857893</x:v>
       </x:c>
       <x:c r="J23" t="str">
         <x:v>2022</x:v>
@@ -2240,7 +2240,7 @@
       </x:c>
       <x:c r="U23" s="8" t="str"/>
       <x:c r="V23" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Golfito%20Golfito%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=8.54636164225735%2C-83.30926901857893</x:v>
       </x:c>
       <x:c r="W23" t="str"/>
       <x:c r="X23" s="8" t="str">
@@ -2253,13 +2253,13 @@
         <x:v>Revisión de alcance, costos, programación y estado del proyecto de sustitución de tuberías y mejoras del sistema dentro del Plan de Inversiones.</x:v>
       </x:c>
       <x:c r="AA23" s="8" t="str">
-        <x:v>Centro urbano de Golfito; no ubicación de obras</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB23" s="8" t="str">
         <x:v>turn6search524</x:v>
       </x:c>
       <x:c r="AC23" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -2285,10 +2285,10 @@
         <x:v>Ciudad Neily</x:v>
       </x:c>
       <x:c r="H24" s="10" t="n">
-        <x:v>8.649</x:v>
+        <x:v>8.64798168958886</x:v>
       </x:c>
       <x:c r="I24" s="10" t="n">
-        <x:v>-82.942</x:v>
+        <x:v>-82.94204922384831</x:v>
       </x:c>
       <x:c r="J24" t="str">
         <x:v>2022</x:v>
@@ -2321,7 +2321,7 @@
       </x:c>
       <x:c r="U24" s="8" t="str"/>
       <x:c r="V24" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Ciudad%20Neily%20Corredores%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=8.64798168958886%2C-82.94204922384831</x:v>
       </x:c>
       <x:c r="W24" t="str"/>
       <x:c r="X24" s="8" t="str">
@@ -2334,13 +2334,13 @@
         <x:v>Revisión de alcance, programación y cartera de inversión para captaciones, planta de tratamiento, bombeo, tanques y líneas de impulsión.</x:v>
       </x:c>
       <x:c r="AA24" s="8" t="str">
-        <x:v>Proyecto extenso Ciudad Neily-Canoas-Laurel-La Cuesta; referencia Ciudad Neily</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB24" s="8" t="str">
         <x:v>turn6search524</x:v>
       </x:c>
       <x:c r="AC24" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2366,10 +2366,10 @@
         <x:v>Ciudad Cortés</x:v>
       </x:c>
       <x:c r="H25" s="10" t="n">
-        <x:v>8.959</x:v>
+        <x:v>8.974381659791892</x:v>
       </x:c>
       <x:c r="I25" s="10" t="n">
-        <x:v>-83.522</x:v>
+        <x:v>-83.52392158218605</x:v>
       </x:c>
       <x:c r="J25" t="str">
         <x:v>2022</x:v>
@@ -2402,7 +2402,7 @@
       </x:c>
       <x:c r="U25" s="8" t="str"/>
       <x:c r="V25" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Ciudad%20Cort%C3%A9s%20Osa%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=8.97438165979189%2C-83.52392158218605</x:v>
       </x:c>
       <x:c r="W25" t="str"/>
       <x:c r="X25" s="8" t="str">
@@ -2415,13 +2415,13 @@
         <x:v>Análisis de información de inversión para planta potabilizadora, almacenamiento, bombeo y líneas de conducción; revisión de costos y programación.</x:v>
       </x:c>
       <x:c r="AA25" s="8" t="str">
-        <x:v>Centro de Ciudad Cortés; obra específica por confirmar</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB25" s="8" t="str">
         <x:v>turn6search524</x:v>
       </x:c>
       <x:c r="AC25" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2447,10 +2447,10 @@
         <x:v>San Ramón / Palmares</x:v>
       </x:c>
       <x:c r="H26" s="10" t="n">
-        <x:v>10.087</x:v>
+        <x:v>10.094727324514901</x:v>
       </x:c>
       <x:c r="I26" s="10" t="n">
-        <x:v>-84.47</x:v>
+        <x:v>-84.4816137876228</x:v>
       </x:c>
       <x:c r="J26" t="str">
         <x:v>2022</x:v>
@@ -2483,7 +2483,7 @@
       </x:c>
       <x:c r="U26" s="8" t="str"/>
       <x:c r="V26" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Ram%C3%B3n%20/%20Palmares%20San%20Ram%C3%B3n%20y%20Palmares%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=10.09472732451490%2C-84.48161378762281</x:v>
       </x:c>
       <x:c r="W26" t="str"/>
       <x:c r="X26" s="8" t="str">
@@ -2496,13 +2496,13 @@
         <x:v>Revisión de factibilidad/diseño, costos y programación para sustitución de redes, separación por niveles de presión y rehabilitación de tanques.</x:v>
       </x:c>
       <x:c r="AA26" s="8" t="str">
-        <x:v>Referencia San Ramón; comprende también Palmares</x:v>
+        <x:v>Coordenada suministrada y revisada por el titular; verificar correspondencia con la obra antes de atribuir una instalación física.</x:v>
       </x:c>
       <x:c r="AB26" s="8" t="str">
         <x:v>turn6search519</x:v>
       </x:c>
       <x:c r="AC26" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2528,10 +2528,10 @@
         <x:v>Puerto Jiménez</x:v>
       </x:c>
       <x:c r="H27" s="10" t="n">
-        <x:v>8.536</x:v>
+        <x:v>8.536945269071543</x:v>
       </x:c>
       <x:c r="I27" s="10" t="n">
-        <x:v>-83.305</x:v>
+        <x:v>-83.30556130171449</x:v>
       </x:c>
       <x:c r="J27" t="str">
         <x:v>2022</x:v>
@@ -2566,7 +2566,7 @@
       </x:c>
       <x:c r="U27" s="8" t="str"/>
       <x:c r="V27" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Puerto%20Jim%C3%A9nez%20Golfito%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=8.53694526907154%2C-83.30556130171449</x:v>
       </x:c>
       <x:c r="W27" t="str"/>
       <x:c r="X27" s="8" t="str">
@@ -2579,13 +2579,13 @@
         <x:v>Revisión de cartera FOPRI y estudios de factibilidad para nuevas fuentes, almacenamiento, distribución de presiones y atención de demanda futura.</x:v>
       </x:c>
       <x:c r="AA27" s="8" t="str">
-        <x:v>Centro de Puerto Jiménez; abarca Bambú y Sándalo</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB27" s="8" t="str">
         <x:v>turn6search507; turn6search519</x:v>
       </x:c>
       <x:c r="AC27" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2611,10 +2611,10 @@
         <x:v>San Pablo de Turrubares</x:v>
       </x:c>
       <x:c r="H28" s="10" t="n">
-        <x:v>9.915</x:v>
+        <x:v>9.908352177656962</x:v>
       </x:c>
       <x:c r="I28" s="10" t="n">
-        <x:v>-84.46</x:v>
+        <x:v>-84.44181429693528</x:v>
       </x:c>
       <x:c r="J28" t="str">
         <x:v>2022</x:v>
@@ -2649,7 +2649,7 @@
       </x:c>
       <x:c r="U28" s="8" t="str"/>
       <x:c r="V28" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Pablo%20de%20Turrubares%20Turrubares%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.90835217765696%2C-84.44181429693528</x:v>
       </x:c>
       <x:c r="W28" t="str"/>
       <x:c r="X28" s="8" t="str">
@@ -2662,13 +2662,13 @@
         <x:v>Revisión de factibilidad, alcance, costos y programación para bombeo, tanque, cloración y ramales hacia comunidades en riesgo sanitario.</x:v>
       </x:c>
       <x:c r="AA28" s="8" t="str">
-        <x:v>Referente poblacional del sistema San Pedro-San Pablo</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB28" s="8" t="str">
         <x:v>turn6search507; turn6search519</x:v>
       </x:c>
       <x:c r="AC28" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2694,10 +2694,10 @@
         <x:v>Colorado de Abangares</x:v>
       </x:c>
       <x:c r="H29" s="10" t="n">
-        <x:v>10.178</x:v>
+        <x:v>10.240034590896785</x:v>
       </x:c>
       <x:c r="I29" s="10" t="n">
-        <x:v>-85.11</x:v>
+        <x:v>-85.10588201384981</x:v>
       </x:c>
       <x:c r="J29" t="str">
         <x:v>2022</x:v>
@@ -2732,7 +2732,7 @@
       </x:c>
       <x:c r="U29" s="8" t="str"/>
       <x:c r="V29" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Colorado%20de%20Abangares%20Abangares%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=10.24003459089679%2C-85.10588201384981</x:v>
       </x:c>
       <x:c r="W29" t="str"/>
       <x:c r="X29" s="8" t="str">
@@ -2745,13 +2745,13 @@
         <x:v>Revisión de información de inversión, costos y programación para incorporación del pozo 3, rehabilitación electromecánica, líneas de impulsión y planta de remoción de hierro y manganeso.</x:v>
       </x:c>
       <x:c r="AA29" s="8" t="str">
-        <x:v>Pueblo de Colorado; pozos y planta no posicionados individualmente</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB29" s="8" t="str">
         <x:v>turn6search507; turn6search519</x:v>
       </x:c>
       <x:c r="AC29" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2777,10 +2777,10 @@
         <x:v>San Isidro de El General</x:v>
       </x:c>
       <x:c r="H30" s="10" t="n">
-        <x:v>9.372</x:v>
+        <x:v>9.3893622580037</x:v>
       </x:c>
       <x:c r="I30" s="10" t="n">
-        <x:v>-83.704</x:v>
+        <x:v>-83.70778394317274</x:v>
       </x:c>
       <x:c r="J30" t="str">
         <x:v>2022</x:v>
@@ -2815,7 +2815,7 @@
         <x:v>https://mapcarta.com/es/San_Isidro_de_El_General</x:v>
       </x:c>
       <x:c r="V30" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Isidro%20de%20El%20General%20Buenos%20Aires%20y%20P%C3%A9rez%20Zeled%C3%B3n%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.38936225800370%2C-83.70778394317274</x:v>
       </x:c>
       <x:c r="W30" t="str"/>
       <x:c r="X30" s="8" t="str">
@@ -2828,13 +2828,13 @@
         <x:v>Seguimiento de proyecto para centralizar parámetros operativos, comunicaciones, registros históricos, alertas y reportes de plantas de tratamiento.</x:v>
       </x:c>
       <x:c r="AA30" s="8" t="str">
-        <x:v>Tres PTAR de la Región Brunca; símbolo orientativo en San Isidro, no las plantas</x:v>
+        <x:v>Coordenada suministrada y revisada por el titular; verificar correspondencia con la obra antes de atribuir una instalación física.</x:v>
       </x:c>
       <x:c r="AB30" s="8" t="str">
         <x:v>turn6search525</x:v>
       </x:c>
       <x:c r="AC30" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2860,10 +2860,10 @@
         <x:v>San Isidro de El General</x:v>
       </x:c>
       <x:c r="H31" s="10" t="n">
-        <x:v>9.372</x:v>
+        <x:v>9.3893622580037</x:v>
       </x:c>
       <x:c r="I31" s="10" t="n">
-        <x:v>-83.704</x:v>
+        <x:v>-83.70778394317274</x:v>
       </x:c>
       <x:c r="J31" t="str">
         <x:v>2022</x:v>
@@ -2898,7 +2898,7 @@
         <x:v>https://mapcarta.com/es/San_Isidro_de_El_General</x:v>
       </x:c>
       <x:c r="V31" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Isidro%20de%20El%20General%20P%C3%A9rez%20Zeled%C3%B3n%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.38936225800370%2C-83.70778394317274</x:v>
       </x:c>
       <x:c r="W31" t="str"/>
       <x:c r="X31" s="8" t="str">
@@ -2911,13 +2911,13 @@
         <x:v>Revisión de programación y costos para estación de bombeo, corrección de colector y trasiego seguro sobre el río San Isidro.</x:v>
       </x:c>
       <x:c r="AA31" s="8" t="str">
-        <x:v>No representa la estación de bombeo en la ribera del río</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB31" s="8" t="str">
         <x:v>turn6search525</x:v>
       </x:c>
       <x:c r="AC31" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2943,10 +2943,10 @@
         <x:v>San Isidro de El General</x:v>
       </x:c>
       <x:c r="H32" s="10" t="n">
-        <x:v>9.372</x:v>
+        <x:v>9.3893622580037</x:v>
       </x:c>
       <x:c r="I32" s="10" t="n">
-        <x:v>-83.704</x:v>
+        <x:v>-83.70778394317274</x:v>
       </x:c>
       <x:c r="J32" t="str">
         <x:v>2022</x:v>
@@ -2981,7 +2981,7 @@
         <x:v>https://mapcarta.com/es/San_Isidro_de_El_General</x:v>
       </x:c>
       <x:c r="V32" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Isidro%20de%20El%20General%20P%C3%A9rez%20Zeled%C3%B3n%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.38936225800370%2C-83.70778394317274</x:v>
       </x:c>
       <x:c r="W32" t="str"/>
       <x:c r="X32" s="8" t="str">
@@ -2994,13 +2994,13 @@
         <x:v>Revisión de cartera y programación para infraestructura de plantel, resguardo de equipo y mejoras de accesos.</x:v>
       </x:c>
       <x:c r="AA32" s="8" t="str">
-        <x:v>Centro urbano, no ubicación precisa de la PTAR</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB32" s="8" t="str">
         <x:v>turn6search525</x:v>
       </x:c>
       <x:c r="AC32" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -3026,10 +3026,10 @@
         <x:v>San José / Periféricos</x:v>
       </x:c>
       <x:c r="H33" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I33" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J33" t="str">
         <x:v>2022</x:v>
@@ -3064,7 +3064,7 @@
       </x:c>
       <x:c r="U33" s="8" t="str"/>
       <x:c r="V33" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Jos%C3%A9%20/%20Perif%C3%A9ricos%20Varios%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W33" t="str"/>
       <x:c r="X33" s="8" t="str">
@@ -3077,13 +3077,13 @@
         <x:v>Preparación de estudios de prefactibilidad, apoyo a supervisión técnica de pozos y conducciones, formulación de proyectos y desarrollo de modelos de datos y tableros para planificación.</x:v>
       </x:c>
       <x:c r="AA33" s="8" t="str">
-        <x:v>Estudios sobre sistemas regionales del país; punto de referencia administrativo</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB33" s="8" t="str">
         <x:v>turn2search442; turn6search563</x:v>
       </x:c>
       <x:c r="AC33" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -3109,10 +3109,10 @@
         <x:v>Río Macho / El Llano</x:v>
       </x:c>
       <x:c r="H34" s="10" t="n">
-        <x:v>9.7654</x:v>
+        <x:v>9.765310222991884</x:v>
       </x:c>
       <x:c r="I34" s="10" t="n">
-        <x:v>-83.8594</x:v>
+        <x:v>-83.85862554910005</x:v>
       </x:c>
       <x:c r="J34" t="str">
         <x:v>2023</x:v>
@@ -3147,7 +3147,7 @@
         <x:v>https://mapcarta.com/W102253746</x:v>
       </x:c>
       <x:c r="V34" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=R%C3%ADo%20Macho%20/%20El%20Llano%20Para%C3%ADso%2C%20El%20Guarco%2C%20Desamparados%2C%20Curridabat%20y%20%C3%A1rea%20metropolitana%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.76531022299188%2C-83.85862554910005</x:v>
       </x:c>
       <x:c r="W34" t="str"/>
       <x:c r="X34" s="8" t="str">
@@ -3160,13 +3160,13 @@
         <x:v>Integración de comisión técnica, revisión del estudio de factibilidad, atención de observaciones MIDEPLAN, homogeneización técnica, marco institucional, población objetivo, costos, cronograma y aspectos de ejecución/operación.</x:v>
       </x:c>
       <x:c r="AA34" s="8" t="str">
-        <x:v>Embalse y ámbito de Río Macho; el PAAM abarca múltiples puntos</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB34" s="8" t="str">
         <x:v>turn2search436; turn6search428; turn6search432; turn6search439; turn6search451</x:v>
       </x:c>
       <x:c r="AC34" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -3192,10 +3192,10 @@
         <x:v>Río Macho / El Llano</x:v>
       </x:c>
       <x:c r="H35" s="10" t="n">
-        <x:v>9.7654</x:v>
+        <x:v>9.765310222991884</x:v>
       </x:c>
       <x:c r="I35" s="10" t="n">
-        <x:v>-83.8594</x:v>
+        <x:v>-83.85862554910005</x:v>
       </x:c>
       <x:c r="J35" t="str">
         <x:v>2023</x:v>
@@ -3230,7 +3230,7 @@
         <x:v>https://mapcarta.com/W102253746</x:v>
       </x:c>
       <x:c r="V35" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=R%C3%ADo%20Macho%20/%20El%20Llano%20Desamparados%20y%20%C3%A1rea%20metropolitana%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.76531022299188%2C-83.85862554910005</x:v>
       </x:c>
       <x:c r="W35" t="str"/>
       <x:c r="X35" s="8" t="str">
@@ -3243,13 +3243,13 @@
         <x:v>Preparación y revisión de fichas descriptivas, estado del proyecto, costos, financiamiento, adquisición de terrenos, cronograma y respuesta para recurso de amparo.</x:v>
       </x:c>
       <x:c r="AA35" s="8" t="str">
-        <x:v>Estudio metropolitano multisitio, no una sola obra</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB35" s="8" t="str">
         <x:v>turn6search429; turn6search431</x:v>
       </x:c>
       <x:c r="AC35" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -3275,10 +3275,10 @@
         <x:v>San Blas / Moravia</x:v>
       </x:c>
       <x:c r="H36" s="10" t="n">
-        <x:v>9.982</x:v>
+        <x:v>9.964014828938442</x:v>
       </x:c>
       <x:c r="I36" s="10" t="n">
-        <x:v>-84.036</x:v>
+        <x:v>-84.03732743593385</x:v>
       </x:c>
       <x:c r="J36" t="str">
         <x:v>2024</x:v>
@@ -3311,7 +3311,7 @@
       </x:c>
       <x:c r="U36" s="8" t="str"/>
       <x:c r="V36" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Blas%20/%20Moravia%20Moravia%2C%20Tib%C3%A1s%20y%20Goicoechea%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.96401482893844%2C-84.03732743593385</x:v>
       </x:c>
       <x:c r="W36" t="str"/>
       <x:c r="X36" s="8" t="str">
@@ -3324,13 +3324,13 @@
         <x:v>Revisión y validación de estado de ejecución, alcance electromecánico, casetas, cloración, extensión eléctrica e interconexiones para mejorar abastecimiento.</x:v>
       </x:c>
       <x:c r="AA36" s="8" t="str">
-        <x:v>Referencia de San Blas; pozo no georreferenciado</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB36" s="8" t="str">
         <x:v>turn6search450</x:v>
       </x:c>
       <x:c r="AC36" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -3356,10 +3356,10 @@
         <x:v>San Jerónimo de Moravia</x:v>
       </x:c>
       <x:c r="H37" s="10" t="n">
-        <x:v>10.012</x:v>
+        <x:v>10.014838896102006</x:v>
       </x:c>
       <x:c r="I37" s="10" t="n">
-        <x:v>-83.973</x:v>
+        <x:v>-83.99757392009057</x:v>
       </x:c>
       <x:c r="J37" t="str">
         <x:v>2024</x:v>
@@ -3392,7 +3392,7 @@
       </x:c>
       <x:c r="U37" s="8" t="str"/>
       <x:c r="V37" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Jer%C3%B3nimo%20de%20Moravia%20V%C3%A1squez%20de%20Coronado%20y%20Moravia%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=10.01483889610201%2C-83.99757392009057</x:v>
       </x:c>
       <x:c r="W37" t="str"/>
       <x:c r="X37" s="8" t="str">
@@ -3405,13 +3405,13 @@
         <x:v>Seguimiento de electrificación de estación de bombeo, operación temporal con generador y estado del proyecto para aumentar el abastecimiento.</x:v>
       </x:c>
       <x:c r="AA37" s="8" t="str">
-        <x:v>Referente de San Jerónimo; captación Río Agra no georreferenciada</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB37" s="8" t="str">
         <x:v>turn6search450</x:v>
       </x:c>
       <x:c r="AC37" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -3437,10 +3437,10 @@
         <x:v>Guadalupe / Goicoechea</x:v>
       </x:c>
       <x:c r="H38" s="10" t="n">
-        <x:v>9.948</x:v>
+        <x:v>9.96408020654612</x:v>
       </x:c>
       <x:c r="I38" s="10" t="n">
-        <x:v>-84.05</x:v>
+        <x:v>-84.0310362737298</x:v>
       </x:c>
       <x:c r="J38" t="str">
         <x:v>2024</x:v>
@@ -3473,7 +3473,7 @@
       </x:c>
       <x:c r="U38" s="8" t="str"/>
       <x:c r="V38" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Guadalupe%20/%20Goicoechea%20Goicoechea%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.96408020654612%2C-84.03103627372980</x:v>
       </x:c>
       <x:c r="W38" t="str"/>
       <x:c r="X38" s="8" t="str">
@@ -3486,13 +3486,13 @@
         <x:v>Seguimiento del pozo perforado, limpieza, armado, prueba de bombeo y búsqueda de recursos para su incorporación al sistema.</x:v>
       </x:c>
       <x:c r="AA38" s="8" t="str">
-        <x:v>Ubicación urbana de Guadalupe; no coordenada del pozo</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB38" s="8" t="str">
         <x:v>turn6search450</x:v>
       </x:c>
       <x:c r="AC38" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -3518,10 +3518,10 @@
         <x:v>GAM</x:v>
       </x:c>
       <x:c r="H39" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I39" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J39" t="str">
         <x:v>2024</x:v>
@@ -3556,7 +3556,7 @@
       </x:c>
       <x:c r="U39" s="8" t="str"/>
       <x:c r="V39" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=GAM%20Varios%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W39" t="str"/>
       <x:c r="X39" s="8" t="str">
@@ -3569,13 +3569,13 @@
         <x:v>Definición de requerimientos prácticos para georradar, calicatas, válvulas, accesorios, comunicación de caudalímetros, coordinación con CCO, inspección, modelación y análisis de mediciones.</x:v>
       </x:c>
       <x:c r="AA39" s="8" t="str">
-        <x:v>Catastro y sectorización en numerosos sistemas; referencia San José</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB39" s="8" t="str">
         <x:v>turn6search448</x:v>
       </x:c>
       <x:c r="AC39" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -3601,10 +3601,10 @@
         <x:v>GAM</x:v>
       </x:c>
       <x:c r="H40" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I40" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J40" t="str">
         <x:v>2025</x:v>
@@ -3637,7 +3637,7 @@
       </x:c>
       <x:c r="U40" s="8" t="str"/>
       <x:c r="V40" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=GAM%20Varios%20cantones%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W40" t="str"/>
       <x:c r="X40" s="8" t="str">
@@ -3650,13 +3650,13 @@
         <x:v>Dirección y elaboración de análisis de demanda, eventos críticos y planes de seguridad del agua para sustentar escenarios y planificación.</x:v>
       </x:c>
       <x:c r="AA40" s="8" t="str">
-        <x:v>Estudio integral, sin un único emplazamiento</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB40" s="8" t="str">
         <x:v>turn6search564</x:v>
       </x:c>
       <x:c r="AC40" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -3682,10 +3682,10 @@
         <x:v>San José (sin sitio publicado)</x:v>
       </x:c>
       <x:c r="H41" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I41" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J41" t="str">
         <x:v>2025</x:v>
@@ -3718,7 +3718,7 @@
       </x:c>
       <x:c r="U41" s="8" t="str"/>
       <x:c r="V41" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Jos%C3%A9%20%28sin%20sitio%20publicado%29%20No%20especificado%20en%20la%20fuente%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W41" t="str"/>
       <x:c r="X41" s="8" t="str">
@@ -3731,13 +3731,13 @@
         <x:v>Dirección del estudio, uso de georradar, análisis de tubería, acceso vial, servidumbre y posibilidad de futuro ramal.</x:v>
       </x:c>
       <x:c r="AA41" s="8" t="str">
-        <x:v>Localización no indicada por la fuente; punto administrativo no corresponde a la propiedad</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB41" s="8" t="str">
         <x:v>turn6search559</x:v>
       </x:c>
       <x:c r="AC41" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -3763,10 +3763,10 @@
         <x:v>Cahuita</x:v>
       </x:c>
       <x:c r="H42" s="10" t="n">
-        <x:v>9.735</x:v>
+        <x:v>9.731571023862829</x:v>
       </x:c>
       <x:c r="I42" s="10" t="n">
-        <x:v>-82.845</x:v>
+        <x:v>-82.84513525696532</x:v>
       </x:c>
       <x:c r="J42" t="str">
         <x:v>2025</x:v>
@@ -3801,7 +3801,7 @@
       </x:c>
       <x:c r="U42" s="8" t="str"/>
       <x:c r="V42" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Cahuita%20Talamanca%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.73157102386283%2C-82.84513525696532</x:v>
       </x:c>
       <x:c r="W42" t="str"/>
       <x:c r="X42" s="8" t="str">
@@ -3814,13 +3814,13 @@
         <x:v>Diagnóstico hidráulico, modelación en período extendido, sectorización, instrumentación, estimación de ANC, comparación IWA/EasyCalc/AWWA, costos de instrumentación y recomendaciones operativas.</x:v>
       </x:c>
       <x:c r="AA42" s="8" t="str">
-        <x:v>Centro de Cahuita; sistema de distribución extenso</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB42" s="8" t="str">
         <x:v>turn2search427; turn6search554</x:v>
       </x:c>
       <x:c r="AC42" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -3846,10 +3846,10 @@
         <x:v>GAM</x:v>
       </x:c>
       <x:c r="H43" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I43" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J43" t="str">
         <x:v>2026</x:v>
@@ -3882,7 +3882,7 @@
       </x:c>
       <x:c r="U43" s="8" t="str"/>
       <x:c r="V43" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=GAM%20Varios%20cantones%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W43" t="str"/>
       <x:c r="X43" s="8" t="str">
@@ -3895,13 +3895,13 @@
         <x:v>Liderazgo en balances oferta-demanda con datos SCADA, aforos, plantas, bombeo, trasvases, facturación, compromisos de caudal y proyectos; elaboración de informe y oficio para Planificación.</x:v>
       </x:c>
       <x:c r="AA43" s="8" t="str">
-        <x:v>Evaluación de numerosos sistemas; no representa una sola obra</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB43" s="8" t="str">
         <x:v>turn1search302; turn6search455</x:v>
       </x:c>
       <x:c r="AC43" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -3927,10 +3927,10 @@
         <x:v>Belén / Puente Mulas</x:v>
       </x:c>
       <x:c r="H44" s="10" t="n">
-        <x:v>9.979</x:v>
+        <x:v>9.972706975052512</x:v>
       </x:c>
       <x:c r="I44" s="10" t="n">
-        <x:v>-84.177</x:v>
+        <x:v>-84.18383232588455</x:v>
       </x:c>
       <x:c r="J44" t="str">
         <x:v>2026</x:v>
@@ -3963,7 +3963,7 @@
       </x:c>
       <x:c r="U44" s="8" t="str"/>
       <x:c r="V44" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Bel%C3%A9n%20/%20Puente%20Mulas%20Bel%C3%A9n%20y%20sectores%20vinculados%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.97270697505251%2C-84.18383232588455</x:v>
       </x:c>
       <x:c r="W44" t="str"/>
       <x:c r="X44" s="8" t="str">
@@ -3976,13 +3976,13 @@
         <x:v>Comparación de fuentes y bombeo, identificación de reducción de producción, análisis de trasvases, déficit, ANC y medidas de recuperación.</x:v>
       </x:c>
       <x:c r="AA44" s="8" t="str">
-        <x:v>Punto representativo del ámbito Puente Mulas</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB44" s="8" t="str">
         <x:v>turn1search302; turn6search455</x:v>
       </x:c>
       <x:c r="AC44" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -4008,10 +4008,10 @@
         <x:v>Santiago de Puriscal</x:v>
       </x:c>
       <x:c r="H45" s="10" t="n">
-        <x:v>9.847</x:v>
+        <x:v>9.849264102346343</x:v>
       </x:c>
       <x:c r="I45" s="10" t="n">
-        <x:v>-84.315</x:v>
+        <x:v>-84.31233506798326</x:v>
       </x:c>
       <x:c r="J45" t="str">
         <x:v>2026</x:v>
@@ -4044,7 +4044,7 @@
       </x:c>
       <x:c r="U45" s="8" t="str"/>
       <x:c r="V45" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Santiago%20de%20Puriscal%20Puriscal%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.84926410234634%2C-84.31233506798326</x:v>
       </x:c>
       <x:c r="W45" t="str"/>
       <x:c r="X45" s="8" t="str">
@@ -4057,13 +4057,13 @@
         <x:v>Dirección de informes, giras y formulación de alternativas sobre fuentes, medición, válvulas, conducciones, almacenamiento, bombeo, sostenibilidad hídrica, terrenos, servidumbres y factibilidad.</x:v>
       </x:c>
       <x:c r="AA45" s="8" t="str">
-        <x:v>Centro cantonal; varias alternativas fuera del casco urbano</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB45" s="8" t="str">
         <x:v>turn2search425; turn6search568; turn6search570</x:v>
       </x:c>
       <x:c r="AC45" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -4089,10 +4089,10 @@
         <x:v>Grifo Alto / Puriscal</x:v>
       </x:c>
       <x:c r="H46" s="10" t="n">
-        <x:v>9.806</x:v>
+        <x:v>9.877536595848015</x:v>
       </x:c>
       <x:c r="I46" s="10" t="n">
-        <x:v>-84.344</x:v>
+        <x:v>-84.3891344534344</x:v>
       </x:c>
       <x:c r="J46" t="str">
         <x:v>2026</x:v>
@@ -4125,7 +4125,7 @@
       </x:c>
       <x:c r="U46" s="8" t="str"/>
       <x:c r="V46" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Grifo%20Alto%20/%20Puriscal%20Puriscal%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.87753659584802%2C-84.38913445343439</x:v>
       </x:c>
       <x:c r="W46" t="str"/>
       <x:c r="X46" s="8" t="str">
@@ -4138,13 +4138,13 @@
         <x:v>Visita técnica, mapas, evaluación de alternativas, revisión de estudio hidráulico 2020, disponibilidad/calidad del pozo, integración al sistema y recomendaciones de formulación y factibilidad.</x:v>
       </x:c>
       <x:c r="AA46" s="8" t="str">
-        <x:v>Referencia de la zona de Grifo Alto; Calle La Máquina por verificar</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB46" s="8" t="str">
         <x:v>turn2search354; turn2search416; turn6search562</x:v>
       </x:c>
       <x:c r="AC46" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -4170,10 +4170,10 @@
         <x:v>GAM</x:v>
       </x:c>
       <x:c r="H47" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I47" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J47" t="str">
         <x:v>2026</x:v>
@@ -4206,7 +4206,7 @@
       </x:c>
       <x:c r="U47" s="8" t="str"/>
       <x:c r="V47" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=GAM%20Varios%20cantones%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W47" t="str"/>
       <x:c r="X47" s="8" t="str">
@@ -4219,13 +4219,13 @@
         <x:v>Autor del cierre técnico y administrativo; revisión de resultados, activos, medición, registro, sistematización, costos, lecciones aprendidas y liquidación técnica.</x:v>
       </x:c>
       <x:c r="AA47" s="8" t="str">
-        <x:v>Proyecto con múltiples caudalímetros; coordenada simbólica</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB47" s="8" t="str">
         <x:v>turn6search574; turn6search455</x:v>
       </x:c>
       <x:c r="AC47" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -4251,10 +4251,10 @@
         <x:v>Guadalupe / Goicoechea</x:v>
       </x:c>
       <x:c r="H48" s="10" t="n">
-        <x:v>9.958</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I48" s="10" t="n">
-        <x:v>-84.051</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J48" t="str">
         <x:v>2026</x:v>
@@ -4287,7 +4287,7 @@
       </x:c>
       <x:c r="U48" s="8" t="str"/>
       <x:c r="V48" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Guadalupe%20/%20Goicoechea%20Goicoechea%2C%20La%20Uni%C3%B3n/Cartago%20y%20Alajuela%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W48" t="str"/>
       <x:c r="X48" s="8" t="str">
@@ -4300,13 +4300,13 @@
         <x:v>Coordinación técnica para sustitución e instalación de caudalímetros, rangos de medición, integración eléctrica, comunicaciones, SCADA y control de producción.</x:v>
       </x:c>
       <x:c r="AA48" s="8" t="str">
-        <x:v>Incluye múltiples instalaciones en Guanacaste, Cartago y Alajuela; símbolo orientativo Guadalupe</x:v>
+        <x:v>Coordenada suministrada y revisada por el titular; verificar correspondencia con la obra antes de atribuir una instalación física.</x:v>
       </x:c>
       <x:c r="AB48" s="8" t="str">
         <x:v>turn6search455</x:v>
       </x:c>
       <x:c r="AC48" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -4332,10 +4332,10 @@
         <x:v>Belén / Fuente Zamora</x:v>
       </x:c>
       <x:c r="H49" s="10" t="n">
-        <x:v>9.979</x:v>
+        <x:v>9.972706975052512</x:v>
       </x:c>
       <x:c r="I49" s="10" t="n">
-        <x:v>-84.177</x:v>
+        <x:v>-84.18383232588455</x:v>
       </x:c>
       <x:c r="J49" t="str">
         <x:v>2026</x:v>
@@ -4368,7 +4368,7 @@
       </x:c>
       <x:c r="U49" s="8" t="str"/>
       <x:c r="V49" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Bel%C3%A9n%20/%20Fuente%20Zamora%20Bel%C3%A9n%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.97270697505251%2C-84.18383232588455</x:v>
       </x:c>
       <x:c r="W49" t="str"/>
       <x:c r="X49" s="8" t="str">
@@ -4381,13 +4381,13 @@
         <x:v>Instalación y puesta en marcha de punto de medición para cuantificar producción, apoyar diagnósticos, sectorización e integración SCADA.</x:v>
       </x:c>
       <x:c r="AA49" s="8" t="str">
-        <x:v>Referencia municipal de la línea PEAD / fuente Zamora</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB49" s="8" t="str">
         <x:v>turn6search455</x:v>
       </x:c>
       <x:c r="AC49" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -4413,10 +4413,10 @@
         <x:v>GAM</x:v>
       </x:c>
       <x:c r="H50" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.913411473518124</x:v>
       </x:c>
       <x:c r="I50" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.12684787186912</x:v>
       </x:c>
       <x:c r="J50" t="str">
         <x:v>2026</x:v>
@@ -4449,7 +4449,7 @@
       </x:c>
       <x:c r="U50" s="8" t="str"/>
       <x:c r="V50" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=GAM%20Varios%20cantones%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.91341147351812%2C-84.12684787186912</x:v>
       </x:c>
       <x:c r="W50" t="str"/>
       <x:c r="X50" s="8" t="str">
@@ -4462,13 +4462,13 @@
         <x:v>Coordinación de modelos hidráulicos, campañas de campo, regulación, monitoreo, válvulas y seguimiento de desempeño.</x:v>
       </x:c>
       <x:c r="AA50" s="8" t="str">
-        <x:v>57 distritos hidrométricos repartidos por la GAM</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB50" s="8" t="str">
         <x:v>turn6search455</x:v>
       </x:c>
       <x:c r="AC50" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -4494,10 +4494,10 @@
         <x:v>Pavas</x:v>
       </x:c>
       <x:c r="H51" s="10" t="n">
-        <x:v>9.947</x:v>
+        <x:v>9.950499992741445</x:v>
       </x:c>
       <x:c r="I51" s="10" t="n">
-        <x:v>-84.141</x:v>
+        <x:v>-84.13916937995353</x:v>
       </x:c>
       <x:c r="J51" t="str">
         <x:v>2026</x:v>
@@ -4530,7 +4530,7 @@
       </x:c>
       <x:c r="U51" s="8" t="str"/>
       <x:c r="V51" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Pavas%20San%20Jos%C3%A9%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.95049999274145%2C-84.13916937995353</x:v>
       </x:c>
       <x:c r="W51" t="str"/>
       <x:c r="X51" s="8" t="str">
@@ -4543,13 +4543,13 @@
         <x:v>Combinación de modelación, mediciones de campo y monitoreo para orientar detección y reparación de fugas no visibles.</x:v>
       </x:c>
       <x:c r="AA51" s="8" t="str">
-        <x:v>Sector Pavas; sin punto de fuga individual</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB51" s="8" t="str">
         <x:v>turn6search455</x:v>
       </x:c>
       <x:c r="AC51" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -4575,10 +4575,10 @@
         <x:v>Alajuelita</x:v>
       </x:c>
       <x:c r="H52" s="10" t="n">
-        <x:v>9.902</x:v>
+        <x:v>9.887104300786469</x:v>
       </x:c>
       <x:c r="I52" s="10" t="n">
-        <x:v>-84.101</x:v>
+        <x:v>-84.10756586210023</x:v>
       </x:c>
       <x:c r="J52" t="str">
         <x:v>2026</x:v>
@@ -4611,7 +4611,7 @@
       </x:c>
       <x:c r="U52" s="8" t="str"/>
       <x:c r="V52" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Alajuelita%20Alajuelita%20y%20cantones%20vinculados%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.88710430078647%2C-84.10756586210023</x:v>
       </x:c>
       <x:c r="W52" t="str"/>
       <x:c r="X52" s="8" t="str">
@@ -4624,13 +4624,13 @@
         <x:v>Preparación de plan con sectores vulnerables, servicios esenciales, almacenamiento, sectorización, presiones, refuerzos y caudales futuros.</x:v>
       </x:c>
       <x:c r="AA52" s="8" t="str">
-        <x:v>Plan de contingencia entre distintos sistemas metropolitanos</x:v>
+        <x:v>Coordenada suministrada y revisada por el titular; verificar correspondencia con la obra antes de atribuir una instalación física.</x:v>
       </x:c>
       <x:c r="AB52" s="8" t="str">
         <x:v>turn2search352; turn6search455</x:v>
       </x:c>
       <x:c r="AC52" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -4656,10 +4656,10 @@
         <x:v>La Unión / San Ramón</x:v>
       </x:c>
       <x:c r="H53" s="10" t="n">
-        <x:v>9.905</x:v>
+        <x:v>9.94922999857834</x:v>
       </x:c>
       <x:c r="I53" s="10" t="n">
-        <x:v>-83.964</x:v>
+        <x:v>-83.96440437290944</x:v>
       </x:c>
       <x:c r="J53" t="str">
         <x:v>2026</x:v>
@@ -4692,7 +4692,7 @@
       </x:c>
       <x:c r="U53" s="8" t="str"/>
       <x:c r="V53" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=La%20Uni%C3%B3n%20/%20San%20Ram%C3%B3n%20La%20Uni%C3%B3n%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.94922999857834%2C-83.96440437290944</x:v>
       </x:c>
       <x:c r="W53" t="str"/>
       <x:c r="X53" s="8" t="str">
@@ -4705,13 +4705,13 @@
         <x:v>Coordinación de instalación de registrador, análisis de continuidad y presiones, diagnóstico estructural, acciones correctivas y plan de cumplimiento de resolución judicial.</x:v>
       </x:c>
       <x:c r="AA53" s="8" t="str">
-        <x:v>Ubicación de referencia para Calle El Cerrito, pendiente identificación puntual</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB53" s="8" t="str">
         <x:v>turn2search381; turn2search398</x:v>
       </x:c>
       <x:c r="AC53" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -4737,10 +4737,10 @@
         <x:v>GAM</x:v>
       </x:c>
       <x:c r="H54" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I54" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J54" t="str">
         <x:v>2026</x:v>
@@ -4773,7 +4773,7 @@
       </x:c>
       <x:c r="U54" s="8" t="str"/>
       <x:c r="V54" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=GAM%20Varios%20cantones%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W54" t="str"/>
       <x:c r="X54" s="8" t="str">
@@ -4786,13 +4786,13 @@
         <x:v>Consolidación, clasificación, agrupamiento por clúster y componentes, depuración de duplicados y preparación de fichas para Planificación y futuros BPIP.</x:v>
       </x:c>
       <x:c r="AA54" s="8" t="str">
-        <x:v>Banco institucional de iniciativas, no una infraestructura física</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB54" s="8" t="str">
         <x:v>turn2search348; turn6search531; turn6search533</x:v>
       </x:c>
       <x:c r="AC54" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -4818,10 +4818,10 @@
         <x:v>San José / institucional</x:v>
       </x:c>
       <x:c r="H55" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I55" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J55" t="str">
         <x:v>2026</x:v>
@@ -4854,7 +4854,7 @@
       </x:c>
       <x:c r="U55" s="8" t="str"/>
       <x:c r="V55" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Jos%C3%A9%20/%20institucional%20No%20aplica%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W55" t="str"/>
       <x:c r="X55" s="8" t="str">
@@ -4867,13 +4867,13 @@
         <x:v>Elaboración de estudio técnico, revisión de admisibilidad, comparación de precios, razonabilidad y recomendación de adjudicación.</x:v>
       </x:c>
       <x:c r="AA55" s="8" t="str">
-        <x:v>Actividad de contratación; símbolo administrativo, no una obra</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB55" s="8" t="str">
         <x:v>turn2search433; turn2search434; turn2search448</x:v>
       </x:c>
       <x:c r="AC55" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -4899,10 +4899,10 @@
         <x:v>San José / alcance nacional</x:v>
       </x:c>
       <x:c r="H56" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I56" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J56" t="str">
         <x:v>2026</x:v>
@@ -4935,7 +4935,7 @@
       </x:c>
       <x:c r="U56" s="8" t="str"/>
       <x:c r="V56" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=San%20Jos%C3%A9%20/%20alcance%20nacional%20Varios%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W56" t="str"/>
       <x:c r="X56" s="8" t="str">
@@ -4948,13 +4948,13 @@
         <x:v>Desarrollo de especificaciones técnicas, evaluación de tecnologías, estudio de mercado, evaluación de ofertas y gestión de contratación.</x:v>
       </x:c>
       <x:c r="AA56" s="8" t="str">
-        <x:v>Licitación institucional con alcance nacional, no localización de obra</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB56" s="8" t="str">
         <x:v>turn2search352; turn6search455</x:v>
       </x:c>
       <x:c r="AC56" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -4980,10 +4980,10 @@
         <x:v>GAM</x:v>
       </x:c>
       <x:c r="H57" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I57" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J57" t="str">
         <x:v>2026</x:v>
@@ -5016,7 +5016,7 @@
       </x:c>
       <x:c r="U57" s="8" t="str"/>
       <x:c r="V57" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=GAM%20Varios%20cantones%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W57" t="str"/>
       <x:c r="X57" s="8" t="str">
@@ -5029,13 +5029,13 @@
         <x:v>Análisis histórico y estratégico de fuentes, almacenamiento, conducciones, retrasos de proyectos y necesidad de hoja de ruta y contingencia para el abastecimiento metropolitano.</x:v>
       </x:c>
       <x:c r="AA57" s="8" t="str">
-        <x:v>Plan de alcance metropolitano; sin sitio único</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB57" s="8" t="str">
         <x:v>turn6search494</x:v>
       </x:c>
       <x:c r="AC57" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -5061,10 +5061,10 @@
         <x:v>GAM / institucional</x:v>
       </x:c>
       <x:c r="H58" s="10" t="n">
-        <x:v>9.9281</x:v>
+        <x:v>9.939163048006971</x:v>
       </x:c>
       <x:c r="I58" s="10" t="n">
-        <x:v>-84.0907</x:v>
+        <x:v>-84.1183104773215</x:v>
       </x:c>
       <x:c r="J58" t="str">
         <x:v>2026</x:v>
@@ -5097,7 +5097,7 @@
       </x:c>
       <x:c r="U58" s="8" t="str"/>
       <x:c r="V58" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=GAM%20/%20institucional%20Varios%20Costa%20Rica</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.93916304800697%2C-84.11831047732150</x:v>
       </x:c>
       <x:c r="W58" t="str"/>
       <x:c r="X58" s="8" t="str">
@@ -5110,13 +5110,13 @@
         <x:v>Apoyo técnico en aplicaciones, georradar, CORS, transición ESRI-Giswater, formularios, integración de datos, bases SQL/PostgreSQL y alternativas de código abierto.</x:v>
       </x:c>
       <x:c r="AA58" s="8" t="str">
-        <x:v>Actividad GIS institucional sin instalación física única</x:v>
+        <x:v>Punto de referencia aportado por el titular. Para programas, estudios o redes multisede no representa necesariamente una instalación puntual.</x:v>
       </x:c>
       <x:c r="AB58" s="8" t="str">
         <x:v>turn6search444; turn6search532</x:v>
       </x:c>
       <x:c r="AC58" t="str">
-        <x:v>Pendiente de coordenada de obra</x:v>
+        <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6907,6 +6907,22 @@
         <x:v>No difundir ubicaciones sensibles de infraestructura de agua ni detalles operativos privados</x:v>
       </x:c>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>Coordenadas actualizadas</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>56 registros actualizados con referencias indicadas por el titular el 2026-10-07; consultar la precisión del proyecto.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>CSP - Brasil (ID 16)</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>La coordenada recibida cae fuera de Ceará. Se mantiene la referencia anterior hasta resolver la discrepancia.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add interactive year timeline and Ricura Walmart project; verify CSP location
</commit_message>
<xml_diff>
--- a/data/proyectos.xlsx
+++ b/data/proyectos.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="1" r:id="Rf99a7e57f13249d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen_42" sheetId="2" r:id="R57eb53133f3d4543"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="3" r:id="Rf3b3ab56fa7b453e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="1" r:id="R723b76bf7423414a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen_42" sheetId="2" r:id="R9c0fa5a03e95460e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="3" r:id="R37dd06980e234154"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,8 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0.000000"/>
+    <x:numFmt numFmtId="201" formatCode="0.000000000000000"/>
   </x:numFmts>
   <x:fonts count="2">
     <x:font>
@@ -55,7 +56,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -80,6 +81,8 @@
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1698,10 +1701,10 @@
         <x:v>Pecém, São Gonçalo do Amarante</x:v>
       </x:c>
       <x:c r="H17" s="10" t="n">
-        <x:v>-3.58535</x:v>
+        <x:v>-3.585917</x:v>
       </x:c>
       <x:c r="I17" s="10" t="n">
-        <x:v>-38.85508</x:v>
+        <x:v>-38.858932</x:v>
       </x:c>
       <x:c r="J17" t="str">
         <x:v>2013</x:v>
@@ -1728,7 +1731,7 @@
         <x:v>Potencia por confirmar</x:v>
       </x:c>
       <x:c r="R17" s="8" t="str">
-        <x:v>Referencia de instalación pública</x:v>
+        <x:v>Coordenada de referencia confirmada por el titular</x:v>
       </x:c>
       <x:c r="S17" t="str">
         <x:v>yes</x:v>
@@ -1740,7 +1743,7 @@
         <x:v>https://www.wikidata.org/wiki/Q18477912</x:v>
       </x:c>
       <x:c r="V17" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Complejo%20sider%C3%BArgico%20CSP%20%E2%80%93%20Brasil%2C%20S%C3%A3o%20Gon%C3%A7alo%20do%20Amarante%2C%20Brasil</x:v>
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=-3.585917%2C-38.858932</x:v>
       </x:c>
       <x:c r="W17" t="str"/>
       <x:c r="X17" s="8" t="str">
@@ -1753,13 +1756,13 @@
         <x:v>Participación en diseño de obras civiles y drenaje</x:v>
       </x:c>
       <x:c r="AA17" s="8" t="str">
-        <x:v>Revisar: la coordenada suministrada (-22.51394179581262, -44.11538570542573) no corresponde a Pecém/Ceará. Se conserva la ubicación anterior de referencia.</x:v>
+        <x:v>Planta siderúrgica CSP, Pecém, Ceará. Coordenada validada por el titular; representa una ubicación de referencia de la instalación.</x:v>
       </x:c>
       <x:c r="AB17" s="8" t="str">
         <x:v>CV 2024/2025/2026</x:v>
       </x:c>
       <x:c r="AC17" t="str">
-        <x:v>PENDIENTE: coordenada suministrada incompatible con Pecém (Ceará). Mantener punto anterior hasta confirmar.</x:v>
+        <x:v>Confirmación del titular, octubre 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -5117,6 +5120,91 @@
       </x:c>
       <x:c r="AC58" t="str">
         <x:v>Coordenada revisada y proporcionada por el titular, 2026-10-07</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="str">
+        <x:v>SCH-RICURA-2015</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>Proyecto</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>Remodelación industrial – Planta Ricura Avícola (Walmart)</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>SCH Consultoría y Construcción / Walmart</x:v>
+      </x:c>
+      <x:c r="E59" t="str">
+        <x:v>Costa Rica</x:v>
+      </x:c>
+      <x:c r="F59" t="str">
+        <x:v>Alajuela</x:v>
+      </x:c>
+      <x:c r="G59" t="str">
+        <x:v>Planta Ricura Avícola</x:v>
+      </x:c>
+      <x:c r="H59" s="17" t="n">
+        <x:v>9.96193965069047</x:v>
+      </x:c>
+      <x:c r="I59" s="17" t="n">
+        <x:v>-84.35572079479125</x:v>
+      </x:c>
+      <x:c r="J59" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="K59" t="str">
+        <x:v>2016</x:v>
+      </x:c>
+      <x:c r="L59" t="str">
+        <x:v>Infraestructura industrial</x:v>
+      </x:c>
+      <x:c r="M59" t="str">
+        <x:v>Finalizado</x:v>
+      </x:c>
+      <x:c r="N59" t="str">
+        <x:v>Ingeniero de proyecto – SCH Consultoría y Construcción</x:v>
+      </x:c>
+      <x:c r="O59" t="str">
+        <x:v>Proyecto principal durante mi etapa en SCH: remodelación de cuartos de refrigeración, mejoras estructurales y trabajos de mantenimiento industrial en la Planta Ricura Avícola de Walmart.</x:v>
+      </x:c>
+      <x:c r="P59" t="str">
+        <x:v>Gestión de proyectos, infraestructura industrial, refrigeración, mantenimiento, obras civiles</x:v>
+      </x:c>
+      <x:c r="Q59" t="str">
+        <x:v>Proyecto principal en SCH</x:v>
+      </x:c>
+      <x:c r="R59" t="str">
+        <x:v>Coordenada verificada por el titular</x:v>
+      </x:c>
+      <x:c r="S59" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="T59" t="str">
+        <x:v>Aporte directo del titular 2026; CV 2025</x:v>
+      </x:c>
+      <x:c r="U59"/>
+      <x:c r="V59" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=9.96193965069047%2C-84.35572079479125</x:v>
+      </x:c>
+      <x:c r="W59"/>
+      <x:c r="X59" t="str">
+        <x:v>Puntual</x:v>
+      </x:c>
+      <x:c r="Y59" t="str">
+        <x:v>Declaración del titular</x:v>
+      </x:c>
+      <x:c r="Z59" t="str">
+        <x:v>Gestión de remodelaciones de cuartos de refrigeración, mejoras estructurales, mantenimiento industrial y coordinación de ejecución durante mi etapa en SCH.</x:v>
+      </x:c>
+      <x:c r="AA59" t="str">
+        <x:v>Coordenadas suministradas y verificadas por el titular para Planta Ricura Avícola (Walmart).</x:v>
+      </x:c>
+      <x:c r="AB59" t="str">
+        <x:v>CV 2025 y aporte del titular</x:v>
+      </x:c>
+      <x:c r="AC59" t="str">
+        <x:v>Coordenada proporcionada y confirmada por el titular, octubre 2026</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>